<commit_message>
fix: RUT_MAP actualizado con clientes faltantes
</commit_message>
<xml_diff>
--- a/datos/Clientes.xlsx
+++ b/datos/Clientes.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/gonpro/Desarrollos/control-despachos/datos/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F5357046-7D9A-D341-B182-6B8A09EF4EA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9BB45EDB-BEA2-264E-985B-12AA8C088E5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12820" yWindow="4340" windowWidth="10000" windowHeight="14260" xr2:uid="{AEC7386F-A211-9841-AA36-A945A6628C87}"/>
+    <workbookView xWindow="6340" yWindow="4340" windowWidth="16480" windowHeight="14260" xr2:uid="{AEC7386F-A211-9841-AA36-A945A6628C87}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="24">
   <si>
     <t>Echeverría Izquierdo Montajes Industriales S.A.</t>
   </si>
@@ -68,9 +68,6 @@
     <t>77.726.289- 0</t>
   </si>
   <si>
-    <t>Tecnasic S.A.</t>
-  </si>
-  <si>
     <t>96.917.120-1</t>
   </si>
   <si>
@@ -102,6 +99,15 @@
   </si>
   <si>
     <t>77.667.046-4</t>
+  </si>
+  <si>
+    <t>Tecnica Nacional De Servicios Ingenieria Y Construccion S.A.</t>
+  </si>
+  <si>
+    <t>Obras Subterráneas S.A. Agencia en Chile</t>
+  </si>
+  <si>
+    <t>76.140.162-9</t>
   </si>
 </sst>
 </file>
@@ -188,7 +194,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -212,6 +218,12 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -549,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{294A12B1-7935-AE42-BABA-9283E4BF5121}">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34.85546875" bestFit="1" customWidth="1"/>
@@ -598,50 +610,58 @@
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B6" s="2" t="s">
         <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="8" t="s">
         <v>12</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" s="4" t="s">
         <v>14</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="B9" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>18</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B11" s="4" t="s">
-        <v>21</v>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>